<commit_message>
fix(gate2): reissue v0.3.1 per gate correction — seals & شناسنامه untouched, CPA→علامتی, real p7-12 content, titles from banners
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/authoring/khshab-G2-MATH_v0.3.1.xlsx
+++ b/authoring/khshab-G2-MATH_v0.3.1.xlsx
@@ -176,7 +176,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -211,7 +211,6 @@
       <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1158,7 +1157,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>در تألیف — v0.3.1 (اصلاحیهٔ گیت موج ۲: بازنویسی ص ۸ تا ۱۲ و Q-1009 تا Q-1024 با محتوای واقعی کتاب؛ بازگشت لایهٔ CPA به «مجسم/تصویری/علامتی»؛ E_GROUPS و E_TABLE_NEIGHBOUR پذیرفته شد؛ موج ۳ فقط پس از سبز شدن v0.3.1)</t>
+          <t>در تألیف — v0.3 (موج ۲: فصل ۱ «عدد و رقم»، ص ۱ تا ۱۸ — ۱۸ ردیف صفحه‌ای + اطلس خطای فصل + بانک سؤال؛ اسکلت موج ۱ (۸ ردیف فصل + فیلدهای کتاب‌محور شناسنامه) تأییدشده و تغییرناپذیر)</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -1678,7 +1677,7 @@
       </c>
       <c r="D7" s="14" t="inlineStr">
         <is>
-          <t>درس ۱: خواندن و مقایسهٔ عدد (تمرین)</t>
+          <t>تمرین (نوع صفحه: تمرین — عنوان بنری مستقل ندارد)</t>
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr">
@@ -1693,7 +1692,7 @@
       </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
-          <t>تمرین: عددنویسی، مقایسه، خواندن از دو طرف</t>
+          <t>تمرین: ساعت، کارت‌های عدد، جای خالی عدد، مقایسه بدون شمردن، عبارت</t>
         </is>
       </c>
       <c r="H7" s="14" t="inlineStr">
@@ -1728,7 +1727,7 @@
       </c>
       <c r="N7" s="14" t="inlineStr">
         <is>
-          <t>شاهد: عکس صفحات ۱ تا ۱۸ (پیوست معلّم) و فایل کتاب C205.pdf — صفحهٔ چاپی ۴.</t>
+          <t>شاهد: عکس معلّم صفحهٔ چاپی ۴ (فایل PDF صفحهٔ ۱۰) + متن PDF — طبق پیام گیت، نوع صفحه «تمرین» است و عنوان بنری مستقل ندارد. محتوا: خواندن ساعت، وصل کردن کارت‌های عدد مثل هم، عدد مناسب در جای خالی، مقایسهٔ بدون شمردن، کامل‌کردن عبارت از دو سو.</t>
         </is>
       </c>
     </row>
@@ -1894,27 +1893,27 @@
       </c>
       <c r="D10" s="14" t="inlineStr">
         <is>
-          <t>درس ۲: تبدیل عدد و رقم (فعّالیت)</t>
+          <t>تمرین (نوع صفحه: تمرین — عنوان بنری مستقل ندارد)</t>
         </is>
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>دانش‌آموز بتواند تعداد دسته‌های ده‌تایی و تک‌ها را به عدد و برعکس تبدیل کند.</t>
+          <t>دانش‌آموز بتواند ادامهٔ عدد ۷۴ را بنویسد، با کارت‌های عدد، عددهای دو رقمی بسازد، جای خالی جدول یکان/دهگان را کامل کند و عدد را به عدد و حروف بنویسد.</t>
         </is>
       </c>
       <c r="F10" s="14" t="inlineStr">
         <is>
-          <t>جدول، عدد، رقم، ده تایی (فقط واژه‌های صفحهٔ ۷)</t>
+          <t>عدد، کارت، جدول، یکان، دهگان (فقط واژه‌های صفحهٔ ۷ از متن PDF و عکس معلّم)</t>
         </is>
       </c>
       <c r="G10" s="14" t="inlineStr">
         <is>
-          <t>فعّالیت: تبدیل دسته‌ها به عدد و بالعکس</t>
+          <t>تمرین: ادامهٔ عدد ۷۴، کارت‌های ۲۴ و ۷، جدول یکان/دهگان، عدد و حروف، الگوی کوچک</t>
         </is>
       </c>
       <c r="H10" s="14" t="inlineStr">
         <is>
-          <t>M_TABLE — جدول یکی/ده‌تایی برای تبدیل بین دسته و عدد</t>
+          <t>M_PLACEVALUE — جدول یکان/دهگان و کارت‌های عدد برای ساختن عدد دو رقمی</t>
         </is>
       </c>
       <c r="I10" s="14" t="inlineStr">
@@ -1944,7 +1943,7 @@
       </c>
       <c r="N10" s="14" t="inlineStr">
         <is>
-          <t>شاهد: عکس صفحات ۱ تا ۱۸ (پیوست معلّم) و فایل کتاب C205.pdf — صفحهٔ چاپی ۷. موتور فعلی بازی ضرب‌محور است؛ اجرای عمیق این فصل نیازمند توسعهٔ متوسط موتور (بسته‌های ده‌تایی/ارزش مکانی) است.</t>
+          <t>شاهد: عکس معلّم صفحهٔ چاپی ۷ (فایل PDF صفحهٔ ۱۳) + متن PDF — طبق پیام گیت، نوع صفحه «تمرین» است و عنوان بنری مستقل ندارد. محتوای دقیق: ادامهٔ عدد ۷۴ (۷۳ تا ۸۰)، کارت‌های ۲۴ و ۷، جدول یکان/دهگان (۵۸، ۶۴، ۱۷)، نوشتن عدد و حروف با رقم‌های ۳ و ۲، ۵ و ۴، ۶ و ۰، عدد دو رقمی با شرط یکان/دهگان، «الگوی کوچک».</t>
         </is>
       </c>
     </row>
@@ -1971,12 +1970,12 @@
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>دانش‌آموز بتواند با کشیدن شکل ساده (مانند مربّع به‌جای کتاب)، مسئله‌های کم‌کردن را حل کند، عدد شکل را بخواند و پنجمین عدد بعد از آن را بنویسد و مجموعه‌ها را از نظر «بیش از ۲۰» مقایسه کند.</t>
+          <t>دانش‌آموز بتواند با کشیدن شکل ساده (مانند مربع به‌جای کتاب)، مسئله‌های کم‌کردن را حل کند، عدد شکل را بخواند و پنجمین عدد بعد از آن را بنویسد و مجموعه‌ها را از نظر «بیش از ۲۰» مقایسه کند.</t>
         </is>
       </c>
       <c r="F11" s="14" t="inlineStr">
         <is>
-          <t>کتاب، علمی، عکس، مربّع، عدد (فقط واژه‌های صفحهٔ ۸ از متن PDF و عکس معلّم)</t>
+          <t>کتاب، علمی، عکس، مربع، عدد (فقط واژه‌های صفحهٔ ۸ از متن PDF و عکس معلّم)</t>
         </is>
       </c>
       <c r="G11" s="14" t="inlineStr">
@@ -1986,7 +1985,7 @@
       </c>
       <c r="H11" s="14" t="inlineStr">
         <is>
-          <t>M_BUNDLES — نمایش ۲۳ کتاب با دو ردیف ده‌تایی مربّع + ۳ تکی؛ شکل‌های ساده به‌جای اشیای مسئله</t>
+          <t>M_BUNDLES — نمایش ۲۳ کتاب با دو ردیف ده‌تایی مربع + ۳ تکی (نمایش دستهٔ ده‌تایی)؛ شکل‌های ساده به‌جای اشیای مسئله</t>
         </is>
       </c>
       <c r="I11" s="14" t="inlineStr">
@@ -2016,7 +2015,7 @@
       </c>
       <c r="N11" s="14" t="inlineStr">
         <is>
-          <t>شاهد: عکس معلّم صفحهٔ ۸ و متن PDF (صفحهٔ ۱۴ فایل) — اعداد دقیق: ۲۳ کتاب (۱۲ داستانی → ۱۱ علمی)، ۳۷ عکس (۲۳ رنگی → ۱۴ سیاه‌وسفید)، شکل مثلث‌ها ۱۶ تا، پنجمین عدد بعد = ۲۱؛ حدس «بیش از ۲۰». موتور فعلی بازی ضرب‌محور است؛ اجرای عمیق این فصل نیازمند توسعهٔ متوسط موتور (بسته‌های ده‌تایی/ارزش مکانی) است.</t>
+          <t>شاهد: عکس معلّم صفحهٔ چاپی ۸ (فایل PDF صفحهٔ ۱۴) + متن PDF — اعداد دقیق: ۲۳ کتاب (۱۲ داستانی → ۱۱ علمی)، ۳۷ عکس (۲۳ رنگی → ۱۴ سیاه‌وسفید)، شکل مثلث‌ها ۱۶ تا، پنجمین عدد بعد = ۲۱؛ «حدس بزن»: مقایسهٔ «بیش از ۲۰» (ملخ‌ها و پروانه‌ها). موتور فعلی بازی ضرب‌محور است؛ اجرای عمیق این فصل نیازمند توسعهٔ متوسط موتور (بسته‌های ده‌تایی/ارزش مکانی) است.</t>
         </is>
       </c>
     </row>
@@ -2043,7 +2042,7 @@
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
-          <t>دانش‌آموز بتواند با پرش روی محور اعداد و ثبت چوب‌خطی، حاصل جمع‌های داستانی (۷+۸ و ۱۲+۵) را به‌دست آورد و قسمت‌های شکل را به‌صورت قرینه کامل کند.</t>
+          <t>دانش‌آموز بتواند با پرش روی محور اعداد و ثبت چوب‌خطی، حاصل جمع‌های داستانی (۷+۸ و ۱۲+۵) را به‌دست آورد و الگوی شکل را در سه قسمت باقی‌مانده کامل کند.</t>
         </is>
       </c>
       <c r="F12" s="14" t="inlineStr">
@@ -2053,12 +2052,12 @@
       </c>
       <c r="G12" s="14" t="inlineStr">
         <is>
-          <t>رسم شکل: پرش روی محور + ثبت چوب‌خطی + کامل کن (قرینه با شابلون)</t>
+          <t>رسم شکل: پرش روی محور تا ۱۶ + ثبت چوب‌خطی + «کامل کن» (کامل‌کردن الگوی شکل — سه قسمت)</t>
         </is>
       </c>
       <c r="H12" s="14" t="inlineStr">
         <is>
-          <t>M_NUMBERLINE — خط اعداد ۰ تا ۱۶ برای پرش ۷+۸؛ ثبت چوب‌خطی ۱۲+۵</t>
+          <t>M_NUMBERLINE — خط اعداد ۰ تا ۱۶ برای پرش ۷+۸ روز؛ ثبت چوب‌خطی ۱۲+۵</t>
         </is>
       </c>
       <c r="I12" s="14" t="inlineStr">
@@ -2088,7 +2087,7 @@
       </c>
       <c r="N12" s="14" t="inlineStr">
         <is>
-          <t>شاهد: عکس معلّم صفحهٔ ۹ و متن PDF (صفحهٔ ۱۵ فایل) — ۷+۸=۱۵ روی خط اعداد تا ۱۶؛ ۱۲+۵=۱۷ با چوب خط؛ جعبهٔ «کامل کن»: تکمیل شکل قرینه با خط‌کش و شابلون (همان «کامل‌کردن الگوی شکل»). موتور فعلی بازی ضرب‌محور است؛ اجرای عمیق این فصل نیازمند توسعهٔ متوسط موتور (بسته‌های ده‌تایی/ارزش مکانی) است.</t>
+          <t>شاهد: عکس معلّم صفحهٔ چاپی ۹ (فایل PDF صفحهٔ ۱۵) + متن PDF — ۷+۸=۱۵ روی خط اعداد تا ۱۶؛ ۱۲+۵=۱۷ با چوب خط؛ بنر جعبه «کامل کن» است: «سه قسمت دیگر شکل را مانند قسمت داده‌شده با خط‌کش و شابلون کامل کنید» — همان «کامل‌کردن الگو (سه‌نمطی)» پیام گیت (سه قسمت باقی‌مانده). موتور فعلی بازی ضرب‌محور است؛ اجرای عمیق این فصل نیازمند توسعهٔ متوسط موتور (بسته‌های ده‌تایی/ارزش مکانی) است.</t>
         </is>
       </c>
     </row>
@@ -2115,22 +2114,22 @@
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>دانش‌آموز بتواند با انگشت، چوب خط، رسم شکل، رنگ‌کردن مربّع‌ها و محور، حاصل جمع و تفریق‌ها و جمع‌های چندجمله‌ای را از راه دلخواه به‌دست آورد.</t>
+          <t>دانش‌آموز بتواند با انگشت، چوب خط، رسم شکل، رنگ‌کردن مربع‌ها و محور اعداد، حاصل جمع و تفریق‌ها و جمع‌های چندجمله‌ای را از راه دلخواه به‌دست آورد.</t>
         </is>
       </c>
       <c r="F13" s="14" t="inlineStr">
         <is>
-          <t>جمع، تفریق، انگشت، چوب خط، مربّع، محور (فقط واژه‌های صفحهٔ ۱۰ از متن PDF و عکس معلّم)</t>
+          <t>جمع، تفریق، انگشت، چوب خط، مربع، محور (فقط واژه‌های صفحهٔ ۱۰ از متن PDF و عکس معلّم)</t>
         </is>
       </c>
       <c r="G13" s="14" t="inlineStr">
         <is>
-          <t>فعّالیت با ۵ روش + کار در کلاس (راه‌های دلخواه)</t>
+          <t>فعّالیت با ۵ روش (انگشت، چوب خط، رسم شکل، رنگ‌آمیزی، محور) + کار در کلاس (راه‌های دلخواه)</t>
         </is>
       </c>
       <c r="H13" s="14" t="inlineStr">
         <is>
-          <t>M_NUMBERLINE — محور برای تفریق‌ها؛ رنگ‌آمیزی مربّع‌ها برای جمع‌ها</t>
+          <t>M_NUMBERLINE — محور اعداد برای تفریق‌ها؛ رنگ‌آمیزی مربع‌ها برای جمع‌ها</t>
         </is>
       </c>
       <c r="I13" s="14" t="inlineStr">
@@ -2160,7 +2159,7 @@
       </c>
       <c r="N13" s="14" t="inlineStr">
         <is>
-          <t>شاهد: عکس معلّم صفحهٔ ۱۰ و متن PDF (صفحهٔ ۱۶ فایل) — عبارت‌های دقیق صفحه: ۴+۳، ۸−۴، ۶+۷، ۸+۹، ۷+۸، ۴+۶+۷، ۳+۴+۵+۶، ۱۲−۷، ۱۵−۷، ۱۳−۹، ۶+۶، ۱۴−۸، ۳+۴، ۷−۵، ۱۱−۵. موتور فعلی بازی ضرب‌محور است؛ اجرای عمیق این فصل نیازمند توسعهٔ متوسط موتور (بسته‌های ده‌تایی/ارزش مکانی) است.</t>
+          <t>شاهد: عکس معلّم صفحهٔ چاپی ۱۰ (فایل PDF صفحهٔ ۱۶) + متن PDF — عبارت‌های دقیق صفحه: ۴+۳، ۸−۴، ۶+۷، ۸+۹، ۷+۸، ۴+۶+۷، ۳+۴+۵+۶، ۱۲−۷، ۱۵−۷، ۱۳−۹، ۶+۶، ۱۴−۸، ۳+۴، ۷−۵، ۱۱−۵. موتور فعلی بازی ضرب‌محور است؛ اجرای عمیق این فصل نیازمند توسعهٔ متوسط موتور (بسته‌های ده‌تایی/ارزش مکانی) است.</t>
         </is>
       </c>
     </row>
@@ -2197,7 +2196,7 @@
       </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
-          <t>فعّالیت دو نفره (مهره) + ادامهٔ الگو + کار در کلاس + حدس بزن (ساعت)</t>
+          <t>فعّالیت دو نفره (مهره) + ادامهٔ الگو + کار در کلاس (جمع‌های چندجمله‌ای) + حدس بزن (ساعت)</t>
         </is>
       </c>
       <c r="H14" s="14" t="inlineStr">
@@ -2232,7 +2231,7 @@
       </c>
       <c r="N14" s="14" t="inlineStr">
         <is>
-          <t>شاهد: عکس معلّم صفحهٔ ۱۱ و متن PDF (صفحهٔ ۱۷ فایل) — بازی با ۷ مهره (تکرار برای ۸، ۹ و ۱۰)؛ الگوها: ۵، ۱۰، ۱۵، ۲۰، … و ۱۰، ۲۰، ۳۰، …؛ جمع‌های چندجمله‌ای: ۱۰+۲۰+۵، ۵+۵+۲۰+۳۰، ۴۰+۵+۱۰+۵+۵، ۱۰+۵+۲۰+۵+۳، ۳+۴+۱۰+۲۰+۵+۵، ۲+۵+۲۰+۱۰+۵، ۱۰+۵+۲۰+۵+۳۰+۵. «حدس بزنِ» خواندن ساعت دست‌ورزی است و بخش تعاملی، جزء و کل و الگوهاست. موتور فعلی بازی ضرب‌محور است؛ اجرای عمیق این فصل نیازمند توسعهٔ متوسط موتور (بسته‌های ده‌تایی/ارزش مکانی) است.</t>
+          <t>شاهد: عکس معلّم صفحهٔ چاپی ۱۱ (فایل PDF صفحهٔ ۱۷) + متن PDF — بازی جزء-کل با ۷ مهره (تکرار برای ۸، ۹ و ۱۰)؛ الگوها: ۵، ۱۰، ۱۵، ۲۰، … و ۱۰، ۲۰، ۳۰، …؛ جمع‌های چندجمله‌ای: ۱۰+۲۰+۵، ۵+۵+۲۰+۳۰، ۴۰+۵+۱۰+۵+۵، ۱۰+۵+۲۰+۵+۳، ۳+۴+۱۰+۲۰+۵+۵، ۲+۵+۲۰+۱۰+۵، ۱۰+۵+۲۰+۵+۳۰+۵. «حدس بزنِ» خواندن ساعت دست‌ورزی است و بخش تعاملی، جزء و کل و الگوهاست. موتور فعلی بازی ضرب‌محور است؛ اجرای عمیق این فصل نیازمند توسعهٔ متوسط موتور (بسته‌های ده‌تایی/ارزش مکانی) است.</t>
         </is>
       </c>
     </row>
@@ -2259,22 +2258,22 @@
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
-          <t>دانش‌آموز بتواند با رنگ‌کردن مربّع‌ها جمع بنویسد، جمع‌های برابر ۷ و برابر ۱۰ را بسازد، حاصل عبارت‌ها را با محور به‌دست آورد و با شابلون ۴ مثلث کنار هم شکل بسازد.</t>
+          <t>دانش‌آموز بتواند با رنگ‌کردن مربع‌ها جمع بنویسد، جمع‌های برابر ۷ و برابر ۱۰ را بسازد، حاصل عبارت‌ها را با محور اعداد به‌دست آورد و با شابلون، مثلث‌ها را کنار هم بکشد.</t>
         </is>
       </c>
       <c r="F15" s="14" t="inlineStr">
         <is>
-          <t>مربّع، رنگ، جمع، محور، مثلث (فقط واژه‌های صفحهٔ ۱۲ از متن PDF و عکس معلّم)</t>
+          <t>مربع، رنگ، جمع، محور، مثلث (فقط واژه‌های صفحهٔ ۱۲ از متن PDF و عکس معلّم)</t>
         </is>
       </c>
       <c r="G15" s="14" t="inlineStr">
         <is>
-          <t>تمرین: رنگ‌آمیزی و نوشتن جمع + محور + خلّق باش (شابلون)</t>
+          <t>تمرین: رنگ‌آمیزی و نوشتن جمع + محاسبه روی محور + «خلاق باش» (شابلون مثلث)</t>
         </is>
       </c>
       <c r="H15" s="14" t="inlineStr">
         <is>
-          <t>M_ARRAY — مربّع‌های رنگی برای جمع‌های برابر ۷ و ۱۰؛ محور اعداد برای ۵+۸ و ۱۳−۸+۷</t>
+          <t>M_ARRAY — مربع‌های رنگی برای جمع‌های برابر ۷ و ۱۰؛ محور اعداد برای ۵+۸ و ۱۳−۸+۷</t>
         </is>
       </c>
       <c r="I15" s="14" t="inlineStr">
@@ -2304,7 +2303,7 @@
       </c>
       <c r="N15" s="14" t="inlineStr">
         <is>
-          <t>شاهد: عکس معلّم صفحهٔ ۱۲ و متن PDF (صفحهٔ ۱۸ فایل) — مثال دقیق: ۵+۲=۷؛ سه‌تایی‌های برابر ۱۰؛ ۵+۸=۱۳ و ۱۳−۸+۷=۱۲ روی محور؛ «خلّق باش»: رسم ۴ مثلث کنار هم با شابلون.</t>
+          <t>شاهد: عکس معلّم صفحهٔ چاپی ۱۲ (فایل PDF صفحهٔ ۱۸) + متن PDF — مثال دقیق: ۵+۲=۷؛ سه‌تایی‌های برابر ۱۰؛ ۵+۸=۱۳ و ۱۳−۸+۷=۱۲ روی محور. بنر جعبه در کتاب «خلاق باش» است («مانند نمونه با استفاده از شابلون مثلث کامل کنید»)؛ در پیام گیت «خطّاپوش» نوشته شده بود — طبق قاعدهٔ «عناوین عیناً از بنر کتاب»، «خلاق باش» ثبت شد.</t>
         </is>
       </c>
     </row>
@@ -2398,12 +2397,12 @@
       </c>
       <c r="D17" s="14" t="inlineStr">
         <is>
-          <t>درس ۵: شمارش سه‌تایی و الگو (فعّالیت)</t>
+          <t>شمارش ۴تا۴تا</t>
         </is>
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t>دانش‌آموز بتواند با شمارش ۳تایی، الگوی رنگی مربع‌ها را ادامه دهد و شکل شابلونی بسازد.</t>
+          <t>دانش‌آموز بتواند با رنگ‌کردن مربع‌ها به‌صورت ۴تایی، الگوی شمارش ۴تایی را کامل کند و روش‌های گوناگون شمارش یک مجموعه را مقایسه کند.</t>
         </is>
       </c>
       <c r="F17" s="14" t="inlineStr">
@@ -2413,12 +2412,12 @@
       </c>
       <c r="G17" s="14" t="inlineStr">
         <is>
-          <t>فعّالیت: شمارش ۳تایی و الگوی رنگی + خلّاق باش</t>
+          <t>فعّالیت: شمارش ۴تا۴تا با رنگ‌آمیزی + کار در کلاس (روش‌های شمارش)</t>
         </is>
       </c>
       <c r="H17" s="14" t="inlineStr">
         <is>
-          <t>M_ARRAY — آرایش مربع‌ها در سطرها برای شمارش چندتایی</t>
+          <t>M_ARRAY — آرایش مربع‌ها در سطرها برای شمارش ۴تا۴تا و کامل‌کردن الگوی شمارش</t>
         </is>
       </c>
       <c r="I17" s="14" t="inlineStr">
@@ -2448,7 +2447,7 @@
       </c>
       <c r="N17" s="14" t="inlineStr">
         <is>
-          <t>شاهد: عکس صفحات ۱ تا ۱۸ (پیوست معلّم) و فایل کتاب C205.pdf — صفحهٔ چاپی ۱۴.</t>
+          <t>شاهد: متن PDF صفحهٔ چاپی ۱۴ + تأیید گیت — «یکی از دانش‌آموزان برای شمارش ۴ تا ۴ تا مربع‌ها را … رنگ کرده»؛ طبق پیام گیت صفحهٔ ۱۴ «شمارش ۴تا۴تا» است (الگوی شمارشِ چندتاییِ v0.3 اصلاح شد).</t>
         </is>
       </c>
     </row>
@@ -2470,7 +2469,7 @@
       </c>
       <c r="D18" s="14" t="inlineStr">
         <is>
-          <t>درس ۵: تمرین‌های شمارش و جمع (تمرین)</t>
+          <t>تمرین (نوع صفحه: تمرین — عنوان بنری مستقل ندارد)</t>
         </is>
       </c>
       <c r="E18" s="14" t="inlineStr">
@@ -2485,7 +2484,7 @@
       </c>
       <c r="G18" s="14" t="inlineStr">
         <is>
-          <t>تمرین: جمع‌ها، عدد قبل/بعد، رنگ‌آمیزی با راهنما</t>
+          <t>تمرین: جمع‌ها با رسم شکل/چوب خط، عدد بعد از ۲۸، عدد قبل از ۴۰، شمارش دایره، رنگ‌آمیزی با راهنما</t>
         </is>
       </c>
       <c r="H18" s="14" t="inlineStr">
@@ -2520,7 +2519,7 @@
       </c>
       <c r="N18" s="14" t="inlineStr">
         <is>
-          <t>شاهد: عکس صفحات ۱ تا ۱۸ (پیوست معلّم) و فایل کتاب C205.pdf — صفحهٔ چاپی ۱۵.</t>
+          <t>شاهد: متن PDF صفحهٔ چاپی ۱۵ + پیام گیت — نوع صفحه «تمرین» است و عنوان بنری مستقل ندارد. محتوا: حاصل جمع‌ها، عدد بعد از ۲۸ (شمارش ۸تایی)، عدد قبل از ۴۰ (شمارش ۵تایی)، شمارش دایره‌ها، رنگ‌آمیزی با راهنما.</t>
         </is>
       </c>
     </row>
@@ -2686,7 +2685,7 @@
       </c>
       <c r="D21" s="14" t="inlineStr">
         <is>
-          <t>معمّا و فرهنگ خواندن</t>
+          <t>معمّا + فرهنگ ریاضی</t>
         </is>
       </c>
       <c r="E21" s="14" t="inlineStr">
@@ -2736,7 +2735,7 @@
       </c>
       <c r="N21" s="14" t="inlineStr">
         <is>
-          <t>شاهد: عکس صفحات ۱ تا ۱۸ (پیوست معلّم) و فایل کتاب C205.pdf — صفحهٔ چاپی ۱۸. رسم مسیر دستی و متن خواندنی است؛ صادقانه «خارج از موتور».</t>
+          <t>شاهد: پیام گیت و صفحهٔ «ساختار کتاب» (نوع فعالیت «فرهنگ ریاضی» در فهرست فعالیت‌های کتاب آمده) — صفحهٔ ۱۸ «معمّا + فرهنگ ریاضی» است و طبق تصریح گیت «خارج از موتور» می‌ماند. (در لایهٔ متن PDF نام «فرهنگ خواندن» آمده بود؛ مرجع نهایی کتاب فیزیکی است.)</t>
         </is>
       </c>
     </row>
@@ -3926,116 +3925,116 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="inlineStr">
+      <c r="A10" s="15" t="inlineStr">
         <is>
           <t>E_GROUPS (پیشنهاد)</t>
         </is>
       </c>
-      <c r="B10" s="16" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>بی‌توجهی به ساختار گروه (کد تازه)</t>
         </is>
       </c>
-      <c r="C10" s="16" t="inlineStr">
+      <c r="C10" s="15" t="inlineStr">
         <is>
           <t>مفهومی</t>
         </is>
       </c>
-      <c r="D10" s="16" t="inlineStr">
+      <c r="D10" s="15" t="inlineStr">
         <is>
           <t>به‌جای شمارش گروه‌ها، تک‌تک می‌شمارد یا فقط تعداد گروه‌ها را می‌نویسد</t>
         </is>
       </c>
-      <c r="E10" s="16" t="inlineStr">
+      <c r="E10" s="15" t="inlineStr">
         <is>
           <t>«۴ دستهٔ ۵تایی» را ۴ یا ۹ می‌نویسد</t>
         </is>
       </c>
-      <c r="F10" s="16" t="inlineStr">
+      <c r="F10" s="15" t="inlineStr">
         <is>
           <t>تصویر گروه‌های برابر + جدول یکی/ده‌تایی</t>
         </is>
       </c>
-      <c r="G10" s="16" t="inlineStr">
+      <c r="G10" s="15" t="inlineStr">
         <is>
           <t>تبدیل گروه به جمع تکراری (۵+۵+۵+۵)؛ ساختن با دستهٔ ده‌تایی</t>
         </is>
       </c>
-      <c r="H10" s="16" t="inlineStr">
+      <c r="H10" s="15" t="inlineStr">
         <is>
           <t>بالا</t>
         </is>
       </c>
-      <c r="I10" s="16" t="inlineStr">
+      <c r="I10" s="15" t="inlineStr">
         <is>
           <t>کد تازه — پیشنهاد AI موتور تألیف v۱.۰</t>
         </is>
       </c>
-      <c r="J10" s="16" t="inlineStr">
-        <is>
-          <t>تأییدشده</t>
-        </is>
-      </c>
-      <c r="K10" s="16" t="inlineStr">
-        <is>
-          <t>کد تازهٔ این موج — همتای مستقیم در errors.js ندارد؛ ستاره‌دار در فصل ۱؛ بیشترین کاربرد: ص ۳، ۸، ۹، ۱۳ — پذیرفته‌شده در گیت موج ۲ (معلّم)؛ پسوند «(پیشنهاد)» برای ثبات شناسه ماند و در نسخهٔ قالب بعدی پاک می‌شود.</t>
+      <c r="J10" s="15" t="inlineStr">
+        <is>
+          <t>نیاز به تأیید</t>
+        </is>
+      </c>
+      <c r="K10" s="15" t="inlineStr">
+        <is>
+          <t>کد تازهٔ این موج — همتای مستقیم در errors.js ندارد؛ ستاره‌دار در فصل ۱؛ بیشترین کاربرد: ص ۳، ۸، ۹، ۱۳</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="16" t="inlineStr">
+      <c r="A11" s="15" t="inlineStr">
         <is>
           <t>E_TABLE_NEIGHBOUR (پیشنهاد)</t>
         </is>
       </c>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr">
         <is>
           <t>اشتباه همسایه‌های جدول (کد تازه)</t>
         </is>
       </c>
-      <c r="C11" s="16" t="inlineStr">
+      <c r="C11" s="15" t="inlineStr">
         <is>
           <t>مفهومی</t>
         </is>
       </c>
-      <c r="D11" s="16" t="inlineStr">
+      <c r="D11" s="15" t="inlineStr">
         <is>
           <t>به‌جای خانهٔ هدف، همسایهٔ بالا/پایین/چپ/راست جدول یا خط اعداد را می‌نویسد</t>
         </is>
       </c>
-      <c r="E11" s="16" t="inlineStr">
+      <c r="E11" s="15" t="inlineStr">
         <is>
           <t>عدد بعد از ۳۹ را ۳۸ یا ۴۹ می‌نویسد</t>
         </is>
       </c>
-      <c r="F11" s="16" t="inlineStr">
+      <c r="F11" s="15" t="inlineStr">
         <is>
           <t>جدول یکی/ده‌تایی یا خط اعداد با یک جای خالی</t>
         </is>
       </c>
-      <c r="G11" s="16" t="inlineStr">
+      <c r="G11" s="15" t="inlineStr">
         <is>
           <t>رنگ‌کردن خانهٔ هدف؛ «همسایه‌ها کدام‌اند؟»</t>
         </is>
       </c>
-      <c r="H11" s="16" t="inlineStr">
+      <c r="H11" s="15" t="inlineStr">
         <is>
           <t>بالا</t>
         </is>
       </c>
-      <c r="I11" s="16" t="inlineStr">
+      <c r="I11" s="15" t="inlineStr">
         <is>
           <t>کد تازه — پیشنهاد AI موتور تألیف v۱.۰</t>
         </is>
       </c>
-      <c r="J11" s="16" t="inlineStr">
-        <is>
-          <t>تأییدشده</t>
-        </is>
-      </c>
-      <c r="K11" s="16" t="inlineStr">
-        <is>
-          <t>کد تازهٔ این موج — ستاره‌دار در فصل ۱؛ بیشترین کاربرد: ص ۵، ۱۰، ۱۲ — پذیرفته‌شده در گیت موج ۲ (معلّم)؛ پسوند «(پیشنهاد)» برای ثبات شناسه ماند و در نسخهٔ قالب بعدی پاک می‌شود.</t>
+      <c r="J11" s="15" t="inlineStr">
+        <is>
+          <t>نیاز به تأیید</t>
+        </is>
+      </c>
+      <c r="K11" s="15" t="inlineStr">
+        <is>
+          <t>کد تازهٔ این موج — ستاره‌دار در فصل ۱؛ بیشترین کاربرد: ص ۵، ۱۰، ۱۲</t>
         </is>
       </c>
     </row>
@@ -4328,7 +4327,7 @@
       </c>
       <c r="D4" s="15" t="inlineStr">
         <is>
-          <t>تصویری</t>
+          <t>علامتی</t>
         </is>
       </c>
       <c r="E4" s="15" t="inlineStr">
@@ -4502,7 +4501,7 @@
       </c>
       <c r="D6" s="15" t="inlineStr">
         <is>
-          <t>تصویری</t>
+          <t>علامتی</t>
         </is>
       </c>
       <c r="E6" s="15" t="inlineStr">
@@ -4589,7 +4588,7 @@
       </c>
       <c r="D7" s="15" t="inlineStr">
         <is>
-          <t>تصویری</t>
+          <t>علامتی</t>
         </is>
       </c>
       <c r="E7" s="15" t="inlineStr">
@@ -5024,7 +5023,7 @@
       </c>
       <c r="D12" s="15" t="inlineStr">
         <is>
-          <t>تصویری</t>
+          <t>علامتی</t>
         </is>
       </c>
       <c r="E12" s="15" t="inlineStr">
@@ -5111,7 +5110,7 @@
       </c>
       <c r="D13" s="15" t="inlineStr">
         <is>
-          <t>تصویری</t>
+          <t>علامتی</t>
         </is>
       </c>
       <c r="E13" s="15" t="inlineStr">
@@ -5198,7 +5197,7 @@
       </c>
       <c r="D14" s="15" t="inlineStr">
         <is>
-          <t>تصویری</t>
+          <t>علامتی</t>
         </is>
       </c>
       <c r="E14" s="15" t="inlineStr">
@@ -5335,7 +5334,7 @@
       </c>
       <c r="N15" s="15" t="inlineStr">
         <is>
-          <t>پاسخ دقیق: ۲۳؛ بقیه کمتر از ۲۰‌اند (حدس بزن صفحهٔ ۸).</t>
+          <t>پاسخ دقیق: ۲۳؛ بقیه کمتر از ۲۰‌اند («حدس بزن» صفحهٔ ۸).</t>
         </is>
       </c>
       <c r="O15" s="15" t="inlineStr">
@@ -5372,7 +5371,7 @@
       </c>
       <c r="D16" s="15" t="inlineStr">
         <is>
-          <t>تصویری</t>
+          <t>علامتی</t>
         </is>
       </c>
       <c r="E16" s="15" t="inlineStr">
@@ -5546,7 +5545,7 @@
       </c>
       <c r="D18" s="15" t="inlineStr">
         <is>
-          <t>تصویری</t>
+          <t>علامتی</t>
         </is>
       </c>
       <c r="E18" s="15" t="inlineStr">
@@ -5981,7 +5980,7 @@
       </c>
       <c r="D23" s="15" t="inlineStr">
         <is>
-          <t>تصویری</t>
+          <t>علامتی</t>
         </is>
       </c>
       <c r="E23" s="15" t="inlineStr">
@@ -6068,7 +6067,7 @@
       </c>
       <c r="D24" s="15" t="inlineStr">
         <is>
-          <t>مجسم</t>
+          <t>علامتی</t>
         </is>
       </c>
       <c r="E24" s="15" t="inlineStr">
@@ -6329,7 +6328,7 @@
       </c>
       <c r="D27" s="15" t="inlineStr">
         <is>
-          <t>مجسم</t>
+          <t>علامتی</t>
         </is>
       </c>
       <c r="E27" s="15" t="inlineStr">
@@ -6503,7 +6502,7 @@
       </c>
       <c r="D29" s="15" t="inlineStr">
         <is>
-          <t>تصویری</t>
+          <t>علامتی</t>
         </is>
       </c>
       <c r="E29" s="15" t="inlineStr">
@@ -6764,7 +6763,7 @@
       </c>
       <c r="D32" s="15" t="inlineStr">
         <is>
-          <t>تصویری</t>
+          <t>علامتی</t>
         </is>
       </c>
       <c r="E32" s="15" t="inlineStr">
@@ -6938,7 +6937,7 @@
       </c>
       <c r="D34" s="15" t="inlineStr">
         <is>
-          <t>تصویری</t>
+          <t>علامتی</t>
         </is>
       </c>
       <c r="E34" s="15" t="inlineStr">
@@ -7460,7 +7459,7 @@
       </c>
       <c r="D40" s="15" t="inlineStr">
         <is>
-          <t>تصویری</t>
+          <t>علامتی</t>
         </is>
       </c>
       <c r="E40" s="15" t="inlineStr">
@@ -7547,7 +7546,7 @@
       </c>
       <c r="D41" s="15" t="inlineStr">
         <is>
-          <t>تصویری</t>
+          <t>علامتی</t>
         </is>
       </c>
       <c r="E41" s="15" t="inlineStr">
@@ -7721,7 +7720,7 @@
       </c>
       <c r="D43" s="15" t="inlineStr">
         <is>
-          <t>تصویری</t>
+          <t>علامتی</t>
         </is>
       </c>
       <c r="E43" s="15" t="inlineStr">

</xml_diff>